<commit_message>
chore: Append real-world backend load testing results to report
</commit_message>
<xml_diff>
--- a/test-reports/Load_Performance_300_TestCases_Analysis_Report.xlsx
+++ b/test-reports/Load_Performance_300_TestCases_Analysis_Report.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55.83203125" customWidth="1" min="1" max="1"/>
@@ -464,7 +464,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -579,7 +578,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -954,6 +952,232 @@
           <t>100.00%</t>
         </is>
       </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RECENT BACKEND LOAD TEST RESULTS (AUTOCANNON)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Target Endpoint</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://cpifzrvgsmoicginrkgj.supabase.co/rest/v1/government_schemes</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Concurrency</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>5 simultaneous connections</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10 seconds</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Latency Metrics</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Value (ms)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Throughput &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Minimum Latency</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>132</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Total Requests</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>56</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Maximum Latency</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>686</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Requests per Second (avg)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Average (Mean)</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>593.6799999999999</v>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Data Transferred</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>56.5 kB</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Median (p50)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>585</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Non-2xx Responses (Errors)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>51</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>90th Percentile (p90)</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>686</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Error Rate</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>99th Percentile (p99)</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>686</v>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Errors likely due to RLS/Rate Limiting</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>